<commit_message>
thumbnail updates, excel template fixes
</commit_message>
<xml_diff>
--- a/content/resources/guides/crate-o/convert-spreadsheet/ro-crate-metadata-template.xlsx
+++ b/content/resources/guides/crate-o/convert-spreadsheet/ro-crate-metadata-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/uqrsmi37/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/uqrsmi37/Documents/Repos/ldaca-website/content/resources/guides/crate-o/convert-spreadsheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2485CD-3C8D-A84E-BAAF-31C6BD6555F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1810098-EB82-8E40-AC5F-49A334190EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="10" r:id="rId1"/>
@@ -18,18 +18,19 @@
     <sheet name="Custom Terms" sheetId="23" r:id="rId3"/>
     <sheet name="Authors" sheetId="12" r:id="rId4"/>
     <sheet name="Publishers" sheetId="11" r:id="rId5"/>
-    <sheet name="Licenses" sheetId="8" r:id="rId6"/>
-    <sheet name="Provenance" sheetId="17" r:id="rId7"/>
-    <sheet name="People" sheetId="7" r:id="rId8"/>
-    <sheet name="Places" sheetId="14" r:id="rId9"/>
-    <sheet name="Localities" sheetId="13" r:id="rId10"/>
-    <sheet name="Objects" sheetId="1" r:id="rId11"/>
-    <sheet name="Files" sheetId="21" r:id="rId12"/>
-    <sheet name="Schemas" sheetId="27" r:id="rId13"/>
-    <sheet name="Columns" sheetId="25" r:id="rId14"/>
+    <sheet name="Languages" sheetId="28" r:id="rId6"/>
+    <sheet name="Licenses" sheetId="8" r:id="rId7"/>
+    <sheet name="Provenance" sheetId="17" r:id="rId8"/>
+    <sheet name="People" sheetId="7" r:id="rId9"/>
+    <sheet name="Places" sheetId="14" r:id="rId10"/>
+    <sheet name="Localities" sheetId="13" r:id="rId11"/>
+    <sheet name="Objects" sheetId="1" r:id="rId12"/>
+    <sheet name="Files" sheetId="21" r:id="rId13"/>
+    <sheet name="Schemas" sheetId="27" r:id="rId14"/>
+    <sheet name="Columns" sheetId="25" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">Objects!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">Objects!$A$1:$K$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="155">
   <si>
     <t>@id</t>
   </si>
@@ -508,6 +509,12 @@
   </si>
   <si>
     <t>asWKT</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>https://glottolog.org/resource/languoid/id/stan1293</t>
   </si>
 </sst>
 </file>
@@ -1191,7 +1198,7 @@
     <xf numFmtId="0" fontId="23" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="30" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="28" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1235,14 +1242,15 @@
     </xf>
     <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="57" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="57" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="58">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1308,6 +1316,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF281160"/>
+      <color rgb="FF150760"/>
       <color rgb="FFE8EAFF"/>
       <color rgb="FFE4E1FF"/>
     </mruColors>
@@ -1624,7 +1634,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.83203125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28.6640625" style="5" bestFit="1" customWidth="1"/>
@@ -1725,16 +1735,18 @@
       <c r="A11" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>47</v>
+      <c r="B11" s="25" t="str">
+        <f>Languages!A2</f>
+        <v>https://glottolog.org/resource/languoid/id/stan1293</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>47</v>
+      <c r="B12" s="25" t="str">
+        <f>Languages!A2</f>
+        <v>https://glottolog.org/resource/languoid/id/stan1293</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -50864,6 +50876,77 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{662AD084-ACEE-B548-980B-57F8B669CD21}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="7" customFormat="1" ht="17" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53972FEC-5747-7342-B007-022E1CF432E7}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -50937,7 +51020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
@@ -51005,7 +51088,7 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="25" t="str">
-        <f>_xlfn.CONCAT("#",C2)</f>
+        <f>_xlfn.CONCAT("#",SUBSTITUTE(C2," ","_"))</f>
         <v>#ExampleCollection_Speaker_01</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -51052,7 +51135,7 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="25" t="str">
-        <f>_xlfn.CONCAT("#",C3)</f>
+        <f>_xlfn.CONCAT("#",SUBSTITUTE(C3," ","_"))</f>
         <v>#ExampleCollection_Speaker_02</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -51333,7 +51416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{048E1B1E-E1A3-DF49-8269-1E379487FFDF}">
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
@@ -51343,7 +51426,7 @@
     <col min="3" max="3" width="28.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32" style="27" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="41" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="11.1640625" style="5"/>
@@ -51365,7 +51448,7 @@
       <c r="E1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="28" t="s">
         <v>33</v>
       </c>
       <c r="G1" s="7" t="s">
@@ -51392,7 +51475,7 @@
       <c r="E2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="31" t="str">
         <f>Objects!A2</f>
         <v>#ExampleCollection_Speaker_01</v>
       </c>
@@ -51416,7 +51499,7 @@
       <c r="E3" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F3" s="31" t="str">
         <f>Objects!A3</f>
         <v>#ExampleCollection_Speaker_02</v>
       </c>
@@ -51440,7 +51523,7 @@
       <c r="E4" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="F4" s="4" t="str">
+      <c r="F4" s="31" t="str">
         <f>Objects!A2</f>
         <v>#ExampleCollection_Speaker_01</v>
       </c>
@@ -51468,7 +51551,7 @@
       <c r="E5" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="31" t="str">
         <f>Objects!A3</f>
         <v>#ExampleCollection_Speaker_02</v>
       </c>
@@ -51494,7 +51577,7 @@
       <c r="E6" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="31" t="str">
         <f>Objects!A2</f>
         <v>#ExampleCollection_Speaker_01</v>
       </c>
@@ -51520,7 +51603,7 @@
       <c r="E7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="31" t="str">
         <f>Objects!A3</f>
         <v>#ExampleCollection_Speaker_02</v>
       </c>
@@ -51538,7 +51621,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B5EE1E-BD49-324F-9063-211D23F5A098}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -51584,7 +51667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{181CD7B9-E188-4741-BCCE-1C7D599060AD}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -51954,6 +52037,41 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5795CE19-579D-C64A-8FE4-5BF2D554C058}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="47.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="7" customFormat="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="5" customFormat="1">
+      <c r="A2" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF0185FB-629C-4D55-88F6-D91170558D6F}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
@@ -52089,7 +52207,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650B96B1-8057-9A43-87CD-EF9ED76014A7}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -52162,7 +52280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABBB93A8-8994-2841-935E-D84C02300906}">
   <dimension ref="A1:F175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
@@ -52670,75 +52788,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{662AD084-ACEE-B548-980B-57F8B669CD21}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="1" width="9.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" s="7" customFormat="1" ht="17" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>